<commit_message>
v54: validation overhaul, logic violations, copy PO fix, feedback alerts
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/reference/dummy_accounts.xlsx
+++ b/reference/dummy_accounts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlo Mauring Lidres\OneDrive\Desktop\Projects\00 Working Projects\ProjectTracker_React\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E275F40-C8ED-4CA7-B8E2-8850A8C94317}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B24768F-E416-422E-8021-514E8B9F9251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4080" yWindow="2220" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>